<commit_message>
2026-09-29 추가 요청 반영 — Mecalac(14개사)·Insight·Benchmarking Report·전문가 피드백·운영 루프
- 경쟁사에 Mecalac 추가(목록·예시·DB 제약·문서), 화면 개수는 목록에서 계산
- 평가 점수 4축(1~5) Schema 추가(v0.2-stage1)
- 07 Insight: 브랜드별 요약·점수 비교·강약점·태그 트렌드·White Space·요약 코멘트(AI 반자동)
- 08 Benchmarking Report: 9개 항목, 인쇄·PDF·xlsx·HTML
- 09 전문가 피드백: 항목·모델별 평가·코멘트·작성자·시각, 반영 상태
- 10 운영 루프: 주기·다음 예정일·오래된 자료 경고·사이클 체크·이력
- 계산은 logic.js, 테스트 60개 / SQL 하네스(기록성 표 칸 단위 GRANT) 통과
- 기획서 v0.2(11장, Proto 13단계 ↔ 메뉴 대응표), 원문·Proto HTML 보관

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/예시데이터_모델목록.xlsx
+++ b/samples/예시데이터_모델목록.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BH15"/>
+  <dimension ref="A1:BL16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -461,123 +461,135 @@
         <v>design_tags</v>
       </c>
       <c r="U1" t="str">
+        <v>score_exterior</v>
+      </c>
+      <c r="V1" t="str">
         <v>glass_area</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>pillar_design</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>visibility</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>console_layout</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>joystick</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>seat</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>display</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>hvac</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AD1" t="str">
+        <v>score_cabin</v>
+      </c>
+      <c r="AE1" t="str">
         <v>main_color</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AF1" t="str">
         <v>accent_color</v>
       </c>
-      <c r="AE1" t="str">
+      <c r="AG1" t="str">
         <v>underbody_color</v>
       </c>
-      <c r="AF1" t="str">
+      <c r="AH1" t="str">
         <v>material</v>
       </c>
-      <c r="AG1" t="str">
+      <c r="AI1" t="str">
         <v>finish</v>
       </c>
-      <c r="AH1" t="str">
+      <c r="AJ1" t="str">
         <v>gloss</v>
       </c>
-      <c r="AI1" t="str">
+      <c r="AK1" t="str">
         <v>texture</v>
       </c>
-      <c r="AJ1" t="str">
+      <c r="AL1" t="str">
+        <v>score_cmf</v>
+      </c>
+      <c r="AM1" t="str">
         <v>operating_weight</v>
       </c>
-      <c r="AK1" t="str">
+      <c r="AN1" t="str">
         <v>engine_power</v>
       </c>
-      <c r="AL1" t="str">
+      <c r="AO1" t="str">
         <v>dimensions</v>
       </c>
-      <c r="AM1" t="str">
+      <c r="AP1" t="str">
         <v>bucket_capacity</v>
       </c>
-      <c r="AN1" t="str">
+      <c r="AQ1" t="str">
         <v>powertrain</v>
       </c>
-      <c r="AO1" t="str">
+      <c r="AR1" t="str">
         <v>maintenance_access</v>
       </c>
-      <c r="AP1" t="str">
+      <c r="AS1" t="str">
         <v>door_parting</v>
       </c>
-      <c r="AQ1" t="str">
+      <c r="AT1" t="str">
         <v>hinge</v>
       </c>
-      <c r="AR1" t="str">
+      <c r="AU1" t="str">
         <v>sensor_camera</v>
       </c>
-      <c r="AS1" t="str">
+      <c r="AV1" t="str">
         <v>safety_label</v>
       </c>
-      <c r="AT1" t="str">
+      <c r="AW1" t="str">
         <v>access</v>
       </c>
-      <c r="AU1" t="str">
+      <c r="AX1" t="str">
+        <v>score_service</v>
+      </c>
+      <c r="AY1" t="str">
         <v>obs_origin</v>
       </c>
-      <c r="AV1" t="str">
+      <c r="AZ1" t="str">
         <v>confidence</v>
       </c>
-      <c r="AW1" t="str">
+      <c r="BA1" t="str">
         <v>extracted_text</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="BB1" t="str">
         <v>evidence_image</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="BC1" t="str">
         <v>human_review_status</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BD1" t="str">
         <v>reviewer_note</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BE1" t="str">
         <v>entered_by</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BF1" t="str">
         <v>prompt_version</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BG1" t="str">
         <v>embedding_id</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BH1" t="str">
         <v>benchmark_scope_id</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BI1" t="str">
         <v>image_path</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BJ1" t="str">
         <v>image_view</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BK1" t="str">
         <v>schema_version</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BL1" t="str">
         <v>id</v>
       </c>
     </row>
@@ -642,18 +654,18 @@
       <c r="T2" t="str">
         <v>저중심 카운터웨이트, 수평 캐릭터라인, 넓은 글라스</v>
       </c>
-      <c r="U2" t="str">
+      <c r="U2">
+        <v>4</v>
+      </c>
+      <c r="V2" t="str">
         <v>넓음(전면 일체형)</v>
       </c>
-      <c r="V2" t="str">
+      <c r="W2" t="str">
         <v>슬림 A필러</v>
       </c>
-      <c r="W2" t="str">
+      <c r="X2" t="str">
         <v>전방·측방 양호</v>
       </c>
-      <c r="X2" t="str">
-        <v/>
-      </c>
       <c r="Y2" t="str">
         <v/>
       </c>
@@ -667,53 +679,53 @@
         <v/>
       </c>
       <c r="AC2" t="str">
+        <v/>
+      </c>
+      <c r="AD2">
+        <v>4</v>
+      </c>
+      <c r="AE2" t="str">
         <v>예시 옐로</v>
       </c>
-      <c r="AD2" t="str">
+      <c r="AF2" t="str">
         <v>다크 그레이</v>
       </c>
-      <c r="AE2" t="str">
+      <c r="AG2" t="str">
         <v>다크 그레이</v>
       </c>
-      <c r="AF2" t="str">
+      <c r="AH2" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG2" t="str">
+      <c r="AI2" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH2" t="str">
+      <c r="AJ2" t="str">
         <v>유광</v>
       </c>
-      <c r="AI2" t="str">
-        <v/>
-      </c>
-      <c r="AJ2">
+      <c r="AK2" t="str">
+        <v/>
+      </c>
+      <c r="AL2">
+        <v>3</v>
+      </c>
+      <c r="AM2">
         <v>21800</v>
       </c>
-      <c r="AK2">
+      <c r="AN2">
         <v>118</v>
       </c>
-      <c r="AL2" t="str">
-        <v/>
-      </c>
-      <c r="AM2">
+      <c r="AO2" t="str">
+        <v/>
+      </c>
+      <c r="AP2">
         <v>1</v>
       </c>
-      <c r="AN2" t="str">
+      <c r="AQ2" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO2" t="str">
+      <c r="AR2" t="str">
         <v>측면 + 상부 점검</v>
       </c>
-      <c r="AP2" t="str">
-        <v/>
-      </c>
-      <c r="AQ2" t="str">
-        <v/>
-      </c>
-      <c r="AR2" t="str">
-        <v/>
-      </c>
       <c r="AS2" t="str">
         <v/>
       </c>
@@ -721,45 +733,57 @@
         <v/>
       </c>
       <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2">
+        <v>4</v>
+      </c>
+      <c r="AY2" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV2" t="str">
-        <v/>
-      </c>
-      <c r="AW2" t="str">
-        <v/>
-      </c>
-      <c r="AX2" t="str">
-        <v/>
-      </c>
-      <c r="AY2" t="str">
+      <c r="AZ2" t="str">
+        <v/>
+      </c>
+      <c r="BA2" t="str">
+        <v/>
+      </c>
+      <c r="BB2" t="str">
+        <v/>
+      </c>
+      <c r="BC2" t="str">
         <v>확정</v>
       </c>
-      <c r="AZ2" t="str">
+      <c r="BD2" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA2" t="str">
+      <c r="BE2" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB2" t="str">
-        <v/>
-      </c>
-      <c r="BC2" t="str">
-        <v/>
-      </c>
-      <c r="BD2" t="str">
-        <v/>
-      </c>
-      <c r="BE2" t="str">
+      <c r="BF2" t="str">
+        <v/>
+      </c>
+      <c r="BG2" t="str">
+        <v/>
+      </c>
+      <c r="BH2" t="str">
+        <v/>
+      </c>
+      <c r="BI2" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF2" t="str">
+      <c r="BJ2" t="str">
         <v>Side; Front-Quarter; Rear; Cabin; CMF Detail</v>
       </c>
-      <c r="BG2" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH2" t="str">
+      <c r="BK2" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL2" t="str">
         <v>M0001</v>
       </c>
     </row>
@@ -824,18 +848,18 @@
       <c r="T3" t="str">
         <v>라운드 후드, 분할형 사이드커버</v>
       </c>
-      <c r="U3" t="str">
+      <c r="U3">
+        <v>3</v>
+      </c>
+      <c r="V3" t="str">
         <v>보통</v>
       </c>
-      <c r="V3" t="str">
+      <c r="W3" t="str">
         <v>일반 A필러</v>
       </c>
-      <c r="W3" t="str">
+      <c r="X3" t="str">
         <v>측방 보통</v>
       </c>
-      <c r="X3" t="str">
-        <v/>
-      </c>
       <c r="Y3" t="str">
         <v/>
       </c>
@@ -849,53 +873,53 @@
         <v/>
       </c>
       <c r="AC3" t="str">
+        <v/>
+      </c>
+      <c r="AD3">
+        <v>3</v>
+      </c>
+      <c r="AE3" t="str">
         <v>예시 블루</v>
       </c>
-      <c r="AD3" t="str">
+      <c r="AF3" t="str">
         <v>차콜</v>
       </c>
-      <c r="AE3" t="str">
+      <c r="AG3" t="str">
         <v>차콜</v>
       </c>
-      <c r="AF3" t="str">
+      <c r="AH3" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG3" t="str">
+      <c r="AI3" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH3" t="str">
+      <c r="AJ3" t="str">
         <v>반광</v>
       </c>
-      <c r="AI3" t="str">
-        <v/>
-      </c>
-      <c r="AJ3">
+      <c r="AK3" t="str">
+        <v/>
+      </c>
+      <c r="AL3">
+        <v>3</v>
+      </c>
+      <c r="AM3">
         <v>22400</v>
       </c>
-      <c r="AK3">
+      <c r="AN3">
         <v>123</v>
       </c>
-      <c r="AL3" t="str">
-        <v/>
-      </c>
-      <c r="AM3">
+      <c r="AO3" t="str">
+        <v/>
+      </c>
+      <c r="AP3">
         <v>1.1</v>
       </c>
-      <c r="AN3" t="str">
+      <c r="AQ3" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO3" t="str">
+      <c r="AR3" t="str">
         <v>측면 지상 점검</v>
       </c>
-      <c r="AP3" t="str">
-        <v/>
-      </c>
-      <c r="AQ3" t="str">
-        <v/>
-      </c>
-      <c r="AR3" t="str">
-        <v/>
-      </c>
       <c r="AS3" t="str">
         <v/>
       </c>
@@ -903,45 +927,57 @@
         <v/>
       </c>
       <c r="AU3" t="str">
+        <v/>
+      </c>
+      <c r="AV3" t="str">
+        <v/>
+      </c>
+      <c r="AW3" t="str">
+        <v/>
+      </c>
+      <c r="AX3">
+        <v>4</v>
+      </c>
+      <c r="AY3" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV3" t="str">
-        <v/>
-      </c>
-      <c r="AW3" t="str">
-        <v/>
-      </c>
-      <c r="AX3" t="str">
-        <v/>
-      </c>
-      <c r="AY3" t="str">
+      <c r="AZ3" t="str">
+        <v/>
+      </c>
+      <c r="BA3" t="str">
+        <v/>
+      </c>
+      <c r="BB3" t="str">
+        <v/>
+      </c>
+      <c r="BC3" t="str">
         <v>미검토</v>
       </c>
-      <c r="AZ3" t="str">
+      <c r="BD3" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA3" t="str">
+      <c r="BE3" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB3" t="str">
-        <v/>
-      </c>
-      <c r="BC3" t="str">
-        <v/>
-      </c>
-      <c r="BD3" t="str">
-        <v/>
-      </c>
-      <c r="BE3" t="str">
+      <c r="BF3" t="str">
+        <v/>
+      </c>
+      <c r="BG3" t="str">
+        <v/>
+      </c>
+      <c r="BH3" t="str">
+        <v/>
+      </c>
+      <c r="BI3" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF3" t="str">
+      <c r="BJ3" t="str">
         <v>Side; Front-Quarter; Cabin; CMF Detail</v>
       </c>
-      <c r="BG3" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH3" t="str">
+      <c r="BK3" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL3" t="str">
         <v>M0002</v>
       </c>
     </row>
@@ -1006,18 +1042,18 @@
       <c r="T4" t="str">
         <v>슬림 필러, 넓은 글라스, 수평 캐릭터라인</v>
       </c>
-      <c r="U4" t="str">
+      <c r="U4">
+        <v>4</v>
+      </c>
+      <c r="V4" t="str">
         <v>넓음(전면 일체형)</v>
       </c>
-      <c r="V4" t="str">
+      <c r="W4" t="str">
         <v>슬림 A필러</v>
       </c>
-      <c r="W4" t="str">
+      <c r="X4" t="str">
         <v>전방·측방 양호</v>
       </c>
-      <c r="X4" t="str">
-        <v/>
-      </c>
       <c r="Y4" t="str">
         <v/>
       </c>
@@ -1031,53 +1067,53 @@
         <v/>
       </c>
       <c r="AC4" t="str">
+        <v/>
+      </c>
+      <c r="AD4">
+        <v>5</v>
+      </c>
+      <c r="AE4" t="str">
         <v>예시 실버</v>
       </c>
-      <c r="AD4" t="str">
+      <c r="AF4" t="str">
         <v>네이비</v>
       </c>
-      <c r="AE4" t="str">
+      <c r="AG4" t="str">
         <v>네이비</v>
       </c>
-      <c r="AF4" t="str">
+      <c r="AH4" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG4" t="str">
+      <c r="AI4" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH4" t="str">
+      <c r="AJ4" t="str">
         <v>유광</v>
       </c>
-      <c r="AI4" t="str">
-        <v/>
-      </c>
-      <c r="AJ4">
+      <c r="AK4" t="str">
+        <v/>
+      </c>
+      <c r="AL4">
+        <v>4</v>
+      </c>
+      <c r="AM4">
         <v>23500</v>
       </c>
-      <c r="AK4">
+      <c r="AN4">
         <v>129</v>
       </c>
-      <c r="AL4" t="str">
-        <v/>
-      </c>
-      <c r="AM4">
+      <c r="AO4" t="str">
+        <v/>
+      </c>
+      <c r="AP4">
         <v>1.2</v>
       </c>
-      <c r="AN4" t="str">
+      <c r="AQ4" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO4" t="str">
+      <c r="AR4" t="str">
         <v>측면 지상 점검</v>
       </c>
-      <c r="AP4" t="str">
-        <v/>
-      </c>
-      <c r="AQ4" t="str">
-        <v/>
-      </c>
-      <c r="AR4" t="str">
-        <v/>
-      </c>
       <c r="AS4" t="str">
         <v/>
       </c>
@@ -1085,45 +1121,57 @@
         <v/>
       </c>
       <c r="AU4" t="str">
+        <v/>
+      </c>
+      <c r="AV4" t="str">
+        <v/>
+      </c>
+      <c r="AW4" t="str">
+        <v/>
+      </c>
+      <c r="AX4">
+        <v>3</v>
+      </c>
+      <c r="AY4" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV4" t="str">
-        <v/>
-      </c>
-      <c r="AW4" t="str">
-        <v/>
-      </c>
-      <c r="AX4" t="str">
-        <v/>
-      </c>
-      <c r="AY4" t="str">
+      <c r="AZ4" t="str">
+        <v/>
+      </c>
+      <c r="BA4" t="str">
+        <v/>
+      </c>
+      <c r="BB4" t="str">
+        <v/>
+      </c>
+      <c r="BC4" t="str">
         <v>미검토</v>
       </c>
-      <c r="AZ4" t="str">
+      <c r="BD4" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA4" t="str">
+      <c r="BE4" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB4" t="str">
-        <v/>
-      </c>
-      <c r="BC4" t="str">
-        <v/>
-      </c>
-      <c r="BD4" t="str">
-        <v/>
-      </c>
-      <c r="BE4" t="str">
+      <c r="BF4" t="str">
+        <v/>
+      </c>
+      <c r="BG4" t="str">
+        <v/>
+      </c>
+      <c r="BH4" t="str">
+        <v/>
+      </c>
+      <c r="BI4" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF4" t="str">
+      <c r="BJ4" t="str">
         <v>Side; Front-Quarter; Rear; Cabin</v>
       </c>
-      <c r="BG4" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH4" t="str">
+      <c r="BK4" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL4" t="str">
         <v>M0003</v>
       </c>
     </row>
@@ -1188,18 +1236,18 @@
       <c r="T5" t="str">
         <v>각진 볼륨, 분할형 사이드커버</v>
       </c>
-      <c r="U5" t="str">
+      <c r="U5">
+        <v>3</v>
+      </c>
+      <c r="V5" t="str">
         <v>보통</v>
       </c>
-      <c r="V5" t="str">
+      <c r="W5" t="str">
         <v>일반 A필러</v>
       </c>
-      <c r="W5" t="str">
+      <c r="X5" t="str">
         <v>측방 보통</v>
       </c>
-      <c r="X5" t="str">
-        <v/>
-      </c>
       <c r="Y5" t="str">
         <v/>
       </c>
@@ -1213,53 +1261,53 @@
         <v/>
       </c>
       <c r="AC5" t="str">
+        <v/>
+      </c>
+      <c r="AD5">
+        <v>3</v>
+      </c>
+      <c r="AE5" t="str">
         <v>예시 오렌지</v>
       </c>
-      <c r="AD5" t="str">
+      <c r="AF5" t="str">
         <v>블랙</v>
       </c>
-      <c r="AE5" t="str">
+      <c r="AG5" t="str">
         <v>블랙</v>
       </c>
-      <c r="AF5" t="str">
+      <c r="AH5" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG5" t="str">
+      <c r="AI5" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH5" t="str">
+      <c r="AJ5" t="str">
         <v>반광</v>
       </c>
-      <c r="AI5" t="str">
-        <v/>
-      </c>
-      <c r="AJ5">
+      <c r="AK5" t="str">
+        <v/>
+      </c>
+      <c r="AL5">
+        <v>3</v>
+      </c>
+      <c r="AM5">
         <v>22000</v>
       </c>
-      <c r="AK5">
+      <c r="AN5">
         <v>122</v>
       </c>
-      <c r="AL5" t="str">
-        <v/>
-      </c>
-      <c r="AM5">
+      <c r="AO5" t="str">
+        <v/>
+      </c>
+      <c r="AP5">
         <v>1</v>
       </c>
-      <c r="AN5" t="str">
+      <c r="AQ5" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO5" t="str">
+      <c r="AR5" t="str">
         <v>측면 + 상부 점검</v>
       </c>
-      <c r="AP5" t="str">
-        <v/>
-      </c>
-      <c r="AQ5" t="str">
-        <v/>
-      </c>
-      <c r="AR5" t="str">
-        <v/>
-      </c>
       <c r="AS5" t="str">
         <v/>
       </c>
@@ -1267,45 +1315,57 @@
         <v/>
       </c>
       <c r="AU5" t="str">
+        <v/>
+      </c>
+      <c r="AV5" t="str">
+        <v/>
+      </c>
+      <c r="AW5" t="str">
+        <v/>
+      </c>
+      <c r="AX5">
+        <v>3</v>
+      </c>
+      <c r="AY5" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV5" t="str">
-        <v/>
-      </c>
-      <c r="AW5" t="str">
-        <v/>
-      </c>
-      <c r="AX5" t="str">
-        <v/>
-      </c>
-      <c r="AY5" t="str">
+      <c r="AZ5" t="str">
+        <v/>
+      </c>
+      <c r="BA5" t="str">
+        <v/>
+      </c>
+      <c r="BB5" t="str">
+        <v/>
+      </c>
+      <c r="BC5" t="str">
         <v>확정</v>
       </c>
-      <c r="AZ5" t="str">
+      <c r="BD5" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA5" t="str">
+      <c r="BE5" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB5" t="str">
-        <v/>
-      </c>
-      <c r="BC5" t="str">
-        <v/>
-      </c>
-      <c r="BD5" t="str">
-        <v/>
-      </c>
-      <c r="BE5" t="str">
+      <c r="BF5" t="str">
+        <v/>
+      </c>
+      <c r="BG5" t="str">
+        <v/>
+      </c>
+      <c r="BH5" t="str">
+        <v/>
+      </c>
+      <c r="BI5" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF5" t="str">
+      <c r="BJ5" t="str">
         <v>Side; Cabin; CMF Detail</v>
       </c>
-      <c r="BG5" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH5" t="str">
+      <c r="BK5" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL5" t="str">
         <v>M0004</v>
       </c>
     </row>
@@ -1370,18 +1430,18 @@
       <c r="T6" t="str">
         <v>각진 볼륨, 저중심 카운터웨이트</v>
       </c>
-      <c r="U6" t="str">
+      <c r="U6">
+        <v>5</v>
+      </c>
+      <c r="V6" t="str">
         <v>보통</v>
       </c>
-      <c r="V6" t="str">
+      <c r="W6" t="str">
         <v>일반 A필러</v>
       </c>
-      <c r="W6" t="str">
+      <c r="X6" t="str">
         <v>측방 보통</v>
       </c>
-      <c r="X6" t="str">
-        <v/>
-      </c>
       <c r="Y6" t="str">
         <v/>
       </c>
@@ -1395,53 +1455,53 @@
         <v/>
       </c>
       <c r="AC6" t="str">
+        <v/>
+      </c>
+      <c r="AD6">
+        <v>3</v>
+      </c>
+      <c r="AE6" t="str">
         <v>예시 옐로</v>
       </c>
-      <c r="AD6" t="str">
+      <c r="AF6" t="str">
         <v>다크 그레이</v>
       </c>
-      <c r="AE6" t="str">
+      <c r="AG6" t="str">
         <v>다크 그레이</v>
       </c>
-      <c r="AF6" t="str">
+      <c r="AH6" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG6" t="str">
+      <c r="AI6" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH6" t="str">
+      <c r="AJ6" t="str">
         <v>유광</v>
       </c>
-      <c r="AI6" t="str">
-        <v/>
-      </c>
-      <c r="AJ6">
+      <c r="AK6" t="str">
+        <v/>
+      </c>
+      <c r="AL6">
+        <v>3</v>
+      </c>
+      <c r="AM6">
         <v>21900</v>
       </c>
-      <c r="AK6">
+      <c r="AN6">
         <v>129</v>
       </c>
-      <c r="AL6" t="str">
-        <v/>
-      </c>
-      <c r="AM6">
+      <c r="AO6" t="str">
+        <v/>
+      </c>
+      <c r="AP6">
         <v>1.1</v>
       </c>
-      <c r="AN6" t="str">
+      <c r="AQ6" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO6" t="str">
+      <c r="AR6" t="str">
         <v>측면 지상 점검</v>
       </c>
-      <c r="AP6" t="str">
-        <v/>
-      </c>
-      <c r="AQ6" t="str">
-        <v/>
-      </c>
-      <c r="AR6" t="str">
-        <v/>
-      </c>
       <c r="AS6" t="str">
         <v/>
       </c>
@@ -1449,45 +1509,57 @@
         <v/>
       </c>
       <c r="AU6" t="str">
+        <v/>
+      </c>
+      <c r="AV6" t="str">
+        <v/>
+      </c>
+      <c r="AW6" t="str">
+        <v/>
+      </c>
+      <c r="AX6">
+        <v>3</v>
+      </c>
+      <c r="AY6" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV6" t="str">
-        <v/>
-      </c>
-      <c r="AW6" t="str">
-        <v/>
-      </c>
-      <c r="AX6" t="str">
-        <v/>
-      </c>
-      <c r="AY6" t="str">
+      <c r="AZ6" t="str">
+        <v/>
+      </c>
+      <c r="BA6" t="str">
+        <v/>
+      </c>
+      <c r="BB6" t="str">
+        <v/>
+      </c>
+      <c r="BC6" t="str">
         <v>미검토</v>
       </c>
-      <c r="AZ6" t="str">
+      <c r="BD6" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA6" t="str">
+      <c r="BE6" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB6" t="str">
-        <v/>
-      </c>
-      <c r="BC6" t="str">
-        <v/>
-      </c>
-      <c r="BD6" t="str">
-        <v/>
-      </c>
-      <c r="BE6" t="str">
+      <c r="BF6" t="str">
+        <v/>
+      </c>
+      <c r="BG6" t="str">
+        <v/>
+      </c>
+      <c r="BH6" t="str">
+        <v/>
+      </c>
+      <c r="BI6" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF6" t="str">
+      <c r="BJ6" t="str">
         <v>Side; Front-Quarter</v>
       </c>
-      <c r="BG6" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH6" t="str">
+      <c r="BK6" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL6" t="str">
         <v>M0005</v>
       </c>
     </row>
@@ -1552,18 +1624,18 @@
       <c r="T7" t="str">
         <v>라운드 후드, 넓은 글라스</v>
       </c>
-      <c r="U7" t="str">
+      <c r="U7">
+        <v>3</v>
+      </c>
+      <c r="V7" t="str">
         <v>넓음(전면 일체형)</v>
       </c>
-      <c r="V7" t="str">
+      <c r="W7" t="str">
         <v>슬림 A필러</v>
       </c>
-      <c r="W7" t="str">
+      <c r="X7" t="str">
         <v>전방·측방 양호</v>
       </c>
-      <c r="X7" t="str">
-        <v/>
-      </c>
       <c r="Y7" t="str">
         <v/>
       </c>
@@ -1577,53 +1649,53 @@
         <v/>
       </c>
       <c r="AC7" t="str">
+        <v/>
+      </c>
+      <c r="AD7">
+        <v>4</v>
+      </c>
+      <c r="AE7" t="str">
         <v>예시 그린</v>
       </c>
-      <c r="AD7" t="str">
+      <c r="AF7" t="str">
         <v>블랙</v>
       </c>
-      <c r="AE7" t="str">
+      <c r="AG7" t="str">
         <v>블랙</v>
       </c>
-      <c r="AF7" t="str">
+      <c r="AH7" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG7" t="str">
+      <c r="AI7" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH7" t="str">
+      <c r="AJ7" t="str">
         <v>반광</v>
       </c>
-      <c r="AI7" t="str">
-        <v/>
-      </c>
-      <c r="AJ7">
+      <c r="AK7" t="str">
+        <v/>
+      </c>
+      <c r="AL7">
+        <v>3</v>
+      </c>
+      <c r="AM7">
         <v>14800</v>
       </c>
-      <c r="AK7">
+      <c r="AN7">
         <v>86</v>
       </c>
-      <c r="AL7" t="str">
-        <v/>
-      </c>
-      <c r="AM7">
+      <c r="AO7" t="str">
+        <v/>
+      </c>
+      <c r="AP7">
         <v>0.6</v>
       </c>
-      <c r="AN7" t="str">
+      <c r="AQ7" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO7" t="str">
+      <c r="AR7" t="str">
         <v>측면 지상 점검</v>
       </c>
-      <c r="AP7" t="str">
-        <v/>
-      </c>
-      <c r="AQ7" t="str">
-        <v/>
-      </c>
-      <c r="AR7" t="str">
-        <v/>
-      </c>
       <c r="AS7" t="str">
         <v/>
       </c>
@@ -1631,45 +1703,57 @@
         <v/>
       </c>
       <c r="AU7" t="str">
+        <v/>
+      </c>
+      <c r="AV7" t="str">
+        <v/>
+      </c>
+      <c r="AW7" t="str">
+        <v/>
+      </c>
+      <c r="AX7">
+        <v>2</v>
+      </c>
+      <c r="AY7" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV7" t="str">
-        <v/>
-      </c>
-      <c r="AW7" t="str">
-        <v/>
-      </c>
-      <c r="AX7" t="str">
-        <v/>
-      </c>
-      <c r="AY7" t="str">
+      <c r="AZ7" t="str">
+        <v/>
+      </c>
+      <c r="BA7" t="str">
+        <v/>
+      </c>
+      <c r="BB7" t="str">
+        <v/>
+      </c>
+      <c r="BC7" t="str">
         <v>미검토</v>
       </c>
-      <c r="AZ7" t="str">
+      <c r="BD7" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA7" t="str">
+      <c r="BE7" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB7" t="str">
-        <v/>
-      </c>
-      <c r="BC7" t="str">
-        <v/>
-      </c>
-      <c r="BD7" t="str">
-        <v/>
-      </c>
-      <c r="BE7" t="str">
+      <c r="BF7" t="str">
+        <v/>
+      </c>
+      <c r="BG7" t="str">
+        <v/>
+      </c>
+      <c r="BH7" t="str">
+        <v/>
+      </c>
+      <c r="BI7" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF7" t="str">
+      <c r="BJ7" t="str">
         <v>Side; Front-Quarter; Cabin; CMF Detail</v>
       </c>
-      <c r="BG7" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH7" t="str">
+      <c r="BK7" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL7" t="str">
         <v>M0006</v>
       </c>
     </row>
@@ -1734,18 +1818,18 @@
       <c r="T8" t="str">
         <v>수평 캐릭터라인</v>
       </c>
-      <c r="U8" t="str">
+      <c r="U8">
+        <v>3</v>
+      </c>
+      <c r="V8" t="str">
         <v>보통</v>
       </c>
-      <c r="V8" t="str">
+      <c r="W8" t="str">
         <v>일반 A필러</v>
       </c>
-      <c r="W8" t="str">
+      <c r="X8" t="str">
         <v>측방 보통</v>
       </c>
-      <c r="X8" t="str">
-        <v/>
-      </c>
       <c r="Y8" t="str">
         <v/>
       </c>
@@ -1759,53 +1843,53 @@
         <v/>
       </c>
       <c r="AC8" t="str">
+        <v/>
+      </c>
+      <c r="AD8">
+        <v>2</v>
+      </c>
+      <c r="AE8" t="str">
         <v>예시 레드</v>
       </c>
-      <c r="AD8" t="str">
+      <c r="AF8" t="str">
         <v>화이트</v>
       </c>
-      <c r="AE8" t="str">
+      <c r="AG8" t="str">
         <v>화이트</v>
       </c>
-      <c r="AF8" t="str">
+      <c r="AH8" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG8" t="str">
+      <c r="AI8" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH8" t="str">
+      <c r="AJ8" t="str">
         <v>유광</v>
       </c>
-      <c r="AI8" t="str">
-        <v/>
-      </c>
-      <c r="AJ8">
+      <c r="AK8" t="str">
+        <v/>
+      </c>
+      <c r="AL8">
+        <v>2</v>
+      </c>
+      <c r="AM8">
         <v>21600</v>
       </c>
-      <c r="AK8">
+      <c r="AN8">
         <v>124</v>
       </c>
-      <c r="AL8" t="str">
-        <v/>
-      </c>
-      <c r="AM8">
+      <c r="AO8" t="str">
+        <v/>
+      </c>
+      <c r="AP8">
         <v>1</v>
       </c>
-      <c r="AN8" t="str">
+      <c r="AQ8" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO8" t="str">
+      <c r="AR8" t="str">
         <v>측면 + 상부 점검</v>
       </c>
-      <c r="AP8" t="str">
-        <v/>
-      </c>
-      <c r="AQ8" t="str">
-        <v/>
-      </c>
-      <c r="AR8" t="str">
-        <v/>
-      </c>
       <c r="AS8" t="str">
         <v/>
       </c>
@@ -1813,45 +1897,57 @@
         <v/>
       </c>
       <c r="AU8" t="str">
+        <v/>
+      </c>
+      <c r="AV8" t="str">
+        <v/>
+      </c>
+      <c r="AW8" t="str">
+        <v/>
+      </c>
+      <c r="AX8">
+        <v>3</v>
+      </c>
+      <c r="AY8" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV8" t="str">
-        <v/>
-      </c>
-      <c r="AW8" t="str">
-        <v/>
-      </c>
-      <c r="AX8" t="str">
-        <v/>
-      </c>
-      <c r="AY8" t="str">
+      <c r="AZ8" t="str">
+        <v/>
+      </c>
+      <c r="BA8" t="str">
+        <v/>
+      </c>
+      <c r="BB8" t="str">
+        <v/>
+      </c>
+      <c r="BC8" t="str">
         <v>확정</v>
       </c>
-      <c r="AZ8" t="str">
+      <c r="BD8" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA8" t="str">
+      <c r="BE8" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB8" t="str">
-        <v/>
-      </c>
-      <c r="BC8" t="str">
-        <v/>
-      </c>
-      <c r="BD8" t="str">
-        <v/>
-      </c>
-      <c r="BE8" t="str">
+      <c r="BF8" t="str">
+        <v/>
+      </c>
+      <c r="BG8" t="str">
+        <v/>
+      </c>
+      <c r="BH8" t="str">
+        <v/>
+      </c>
+      <c r="BI8" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF8" t="str">
+      <c r="BJ8" t="str">
         <v>Side; CMF Detail</v>
       </c>
-      <c r="BG8" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH8" t="str">
+      <c r="BK8" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL8" t="str">
         <v>M0007</v>
       </c>
     </row>
@@ -1916,18 +2012,18 @@
       <c r="T9" t="str">
         <v>각진 볼륨</v>
       </c>
-      <c r="U9" t="str">
+      <c r="U9">
+        <v>4</v>
+      </c>
+      <c r="V9" t="str">
         <v>보통</v>
       </c>
-      <c r="V9" t="str">
+      <c r="W9" t="str">
         <v>일반 A필러</v>
       </c>
-      <c r="W9" t="str">
+      <c r="X9" t="str">
         <v>측방 보통</v>
       </c>
-      <c r="X9" t="str">
-        <v/>
-      </c>
       <c r="Y9" t="str">
         <v/>
       </c>
@@ -1941,53 +2037,53 @@
         <v/>
       </c>
       <c r="AC9" t="str">
+        <v/>
+      </c>
+      <c r="AD9">
+        <v>2</v>
+      </c>
+      <c r="AE9" t="str">
         <v>예시 오렌지</v>
       </c>
-      <c r="AD9" t="str">
+      <c r="AF9" t="str">
         <v>블랙</v>
       </c>
-      <c r="AE9" t="str">
+      <c r="AG9" t="str">
         <v>블랙</v>
       </c>
-      <c r="AF9" t="str">
+      <c r="AH9" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG9" t="str">
+      <c r="AI9" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH9" t="str">
+      <c r="AJ9" t="str">
         <v>반광</v>
       </c>
-      <c r="AI9" t="str">
-        <v/>
-      </c>
-      <c r="AJ9">
+      <c r="AK9" t="str">
+        <v/>
+      </c>
+      <c r="AL9">
+        <v>3</v>
+      </c>
+      <c r="AM9">
         <v>22100</v>
       </c>
-      <c r="AK9">
+      <c r="AN9">
         <v>118</v>
       </c>
-      <c r="AL9" t="str">
-        <v/>
-      </c>
-      <c r="AM9">
+      <c r="AO9" t="str">
+        <v/>
+      </c>
+      <c r="AP9">
         <v>1.1</v>
       </c>
-      <c r="AN9" t="str">
+      <c r="AQ9" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO9" t="str">
+      <c r="AR9" t="str">
         <v>측면 지상 점검</v>
       </c>
-      <c r="AP9" t="str">
-        <v/>
-      </c>
-      <c r="AQ9" t="str">
-        <v/>
-      </c>
-      <c r="AR9" t="str">
-        <v/>
-      </c>
       <c r="AS9" t="str">
         <v/>
       </c>
@@ -1995,45 +2091,57 @@
         <v/>
       </c>
       <c r="AU9" t="str">
+        <v/>
+      </c>
+      <c r="AV9" t="str">
+        <v/>
+      </c>
+      <c r="AW9" t="str">
+        <v/>
+      </c>
+      <c r="AX9">
+        <v>3</v>
+      </c>
+      <c r="AY9" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV9" t="str">
-        <v/>
-      </c>
-      <c r="AW9" t="str">
-        <v/>
-      </c>
-      <c r="AX9" t="str">
-        <v/>
-      </c>
-      <c r="AY9" t="str">
+      <c r="AZ9" t="str">
+        <v/>
+      </c>
+      <c r="BA9" t="str">
+        <v/>
+      </c>
+      <c r="BB9" t="str">
+        <v/>
+      </c>
+      <c r="BC9" t="str">
         <v>미검토</v>
       </c>
-      <c r="AZ9" t="str">
+      <c r="BD9" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA9" t="str">
+      <c r="BE9" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB9" t="str">
-        <v/>
-      </c>
-      <c r="BC9" t="str">
-        <v/>
-      </c>
-      <c r="BD9" t="str">
-        <v/>
-      </c>
-      <c r="BE9" t="str">
+      <c r="BF9" t="str">
+        <v/>
+      </c>
+      <c r="BG9" t="str">
+        <v/>
+      </c>
+      <c r="BH9" t="str">
+        <v/>
+      </c>
+      <c r="BI9" t="str">
         <v>(브라우저 보관 이미지)</v>
       </c>
-      <c r="BF9" t="str">
+      <c r="BJ9" t="str">
         <v>Side</v>
       </c>
-      <c r="BG9" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH9" t="str">
+      <c r="BK9" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL9" t="str">
         <v>M0008</v>
       </c>
     </row>
@@ -2098,18 +2206,18 @@
       <c r="T10" t="str">
         <v>후방 소선회, 라운드 후드</v>
       </c>
-      <c r="U10" t="str">
+      <c r="U10">
+        <v>3</v>
+      </c>
+      <c r="V10" t="str">
         <v>보통</v>
       </c>
-      <c r="V10" t="str">
+      <c r="W10" t="str">
         <v>일반 A필러</v>
       </c>
-      <c r="W10" t="str">
+      <c r="X10" t="str">
         <v>측방 보통</v>
       </c>
-      <c r="X10" t="str">
-        <v/>
-      </c>
       <c r="Y10" t="str">
         <v/>
       </c>
@@ -2123,53 +2231,53 @@
         <v/>
       </c>
       <c r="AC10" t="str">
+        <v/>
+      </c>
+      <c r="AD10">
+        <v>3</v>
+      </c>
+      <c r="AE10" t="str">
         <v>예시 레드</v>
       </c>
-      <c r="AD10" t="str">
+      <c r="AF10" t="str">
         <v>화이트</v>
       </c>
-      <c r="AE10" t="str">
+      <c r="AG10" t="str">
         <v>화이트</v>
       </c>
-      <c r="AF10" t="str">
+      <c r="AH10" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG10" t="str">
+      <c r="AI10" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH10" t="str">
+      <c r="AJ10" t="str">
         <v>유광</v>
       </c>
-      <c r="AI10" t="str">
-        <v/>
-      </c>
-      <c r="AJ10">
+      <c r="AK10" t="str">
+        <v/>
+      </c>
+      <c r="AL10">
+        <v>3</v>
+      </c>
+      <c r="AM10">
         <v>3600</v>
       </c>
-      <c r="AK10">
+      <c r="AN10">
         <v>18</v>
       </c>
-      <c r="AL10" t="str">
-        <v/>
-      </c>
-      <c r="AM10">
+      <c r="AO10" t="str">
+        <v/>
+      </c>
+      <c r="AP10">
         <v>0.1</v>
       </c>
-      <c r="AN10" t="str">
+      <c r="AQ10" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO10" t="str">
+      <c r="AR10" t="str">
         <v>측면 지상 점검</v>
       </c>
-      <c r="AP10" t="str">
-        <v/>
-      </c>
-      <c r="AQ10" t="str">
-        <v/>
-      </c>
-      <c r="AR10" t="str">
-        <v/>
-      </c>
       <c r="AS10" t="str">
         <v/>
       </c>
@@ -2177,45 +2285,57 @@
         <v/>
       </c>
       <c r="AU10" t="str">
+        <v/>
+      </c>
+      <c r="AV10" t="str">
+        <v/>
+      </c>
+      <c r="AW10" t="str">
+        <v/>
+      </c>
+      <c r="AX10">
+        <v>4</v>
+      </c>
+      <c r="AY10" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV10" t="str">
-        <v/>
-      </c>
-      <c r="AW10" t="str">
-        <v/>
-      </c>
-      <c r="AX10" t="str">
-        <v/>
-      </c>
-      <c r="AY10" t="str">
+      <c r="AZ10" t="str">
+        <v/>
+      </c>
+      <c r="BA10" t="str">
+        <v/>
+      </c>
+      <c r="BB10" t="str">
+        <v/>
+      </c>
+      <c r="BC10" t="str">
         <v>미검토</v>
       </c>
-      <c r="AZ10" t="str">
+      <c r="BD10" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA10" t="str">
+      <c r="BE10" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB10" t="str">
-        <v/>
-      </c>
-      <c r="BC10" t="str">
-        <v/>
-      </c>
-      <c r="BD10" t="str">
-        <v/>
-      </c>
-      <c r="BE10" t="str">
+      <c r="BF10" t="str">
+        <v/>
+      </c>
+      <c r="BG10" t="str">
+        <v/>
+      </c>
+      <c r="BH10" t="str">
+        <v/>
+      </c>
+      <c r="BI10" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF10" t="str">
+      <c r="BJ10" t="str">
         <v>Side; Front-Quarter; Cabin</v>
       </c>
-      <c r="BG10" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH10" t="str">
+      <c r="BK10" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL10" t="str">
         <v>M0009</v>
       </c>
     </row>
@@ -2281,17 +2401,17 @@
         <v>후방 소선회</v>
       </c>
       <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
         <v>보통</v>
       </c>
-      <c r="V11" t="str">
+      <c r="W11" t="str">
         <v>일반 A필러</v>
       </c>
-      <c r="W11" t="str">
+      <c r="X11" t="str">
         <v>측방 보통</v>
       </c>
-      <c r="X11" t="str">
-        <v/>
-      </c>
       <c r="Y11" t="str">
         <v/>
       </c>
@@ -2305,53 +2425,53 @@
         <v/>
       </c>
       <c r="AC11" t="str">
+        <v/>
+      </c>
+      <c r="AD11" t="str">
+        <v/>
+      </c>
+      <c r="AE11" t="str">
         <v>예시 블루</v>
       </c>
-      <c r="AD11" t="str">
+      <c r="AF11" t="str">
         <v>차콜</v>
       </c>
-      <c r="AE11" t="str">
+      <c r="AG11" t="str">
         <v>차콜</v>
       </c>
-      <c r="AF11" t="str">
+      <c r="AH11" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG11" t="str">
+      <c r="AI11" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH11" t="str">
+      <c r="AJ11" t="str">
         <v>반광</v>
       </c>
-      <c r="AI11" t="str">
-        <v/>
-      </c>
-      <c r="AJ11">
+      <c r="AK11" t="str">
+        <v/>
+      </c>
+      <c r="AL11" t="str">
+        <v/>
+      </c>
+      <c r="AM11">
         <v>3100</v>
       </c>
-      <c r="AK11">
+      <c r="AN11">
         <v>16</v>
       </c>
-      <c r="AL11" t="str">
-        <v/>
-      </c>
-      <c r="AM11">
+      <c r="AO11" t="str">
+        <v/>
+      </c>
+      <c r="AP11">
         <v>0.09</v>
       </c>
-      <c r="AN11" t="str">
+      <c r="AQ11" t="str">
         <v>디젤 (예시)</v>
       </c>
-      <c r="AO11" t="str">
+      <c r="AR11" t="str">
         <v>측면 + 상부 점검</v>
       </c>
-      <c r="AP11" t="str">
-        <v/>
-      </c>
-      <c r="AQ11" t="str">
-        <v/>
-      </c>
-      <c r="AR11" t="str">
-        <v/>
-      </c>
       <c r="AS11" t="str">
         <v/>
       </c>
@@ -2359,45 +2479,57 @@
         <v/>
       </c>
       <c r="AU11" t="str">
+        <v/>
+      </c>
+      <c r="AV11" t="str">
+        <v/>
+      </c>
+      <c r="AW11" t="str">
+        <v/>
+      </c>
+      <c r="AX11" t="str">
+        <v/>
+      </c>
+      <c r="AY11" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV11" t="str">
-        <v/>
-      </c>
-      <c r="AW11" t="str">
-        <v/>
-      </c>
-      <c r="AX11" t="str">
-        <v/>
-      </c>
-      <c r="AY11" t="str">
+      <c r="AZ11" t="str">
+        <v/>
+      </c>
+      <c r="BA11" t="str">
+        <v/>
+      </c>
+      <c r="BB11" t="str">
+        <v/>
+      </c>
+      <c r="BC11" t="str">
         <v>확정</v>
       </c>
-      <c r="AZ11" t="str">
+      <c r="BD11" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA11" t="str">
+      <c r="BE11" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB11" t="str">
-        <v/>
-      </c>
-      <c r="BC11" t="str">
-        <v/>
-      </c>
-      <c r="BD11" t="str">
-        <v/>
-      </c>
-      <c r="BE11" t="str">
+      <c r="BF11" t="str">
+        <v/>
+      </c>
+      <c r="BG11" t="str">
+        <v/>
+      </c>
+      <c r="BH11" t="str">
+        <v/>
+      </c>
+      <c r="BI11" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF11" t="str">
+      <c r="BJ11" t="str">
         <v>Side; CMF Detail</v>
       </c>
-      <c r="BG11" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH11" t="str">
+      <c r="BK11" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL11" t="str">
         <v>M0010</v>
       </c>
     </row>
@@ -2462,18 +2594,18 @@
       <c r="T12" t="str">
         <v>후방 경사 후드, 넓은 글라스</v>
       </c>
-      <c r="U12" t="str">
+      <c r="U12">
+        <v>4</v>
+      </c>
+      <c r="V12" t="str">
         <v>넓음(전면 일체형)</v>
       </c>
-      <c r="V12" t="str">
+      <c r="W12" t="str">
         <v>슬림 A필러</v>
       </c>
-      <c r="W12" t="str">
+      <c r="X12" t="str">
         <v>전방·측방 양호</v>
       </c>
-      <c r="X12" t="str">
-        <v/>
-      </c>
       <c r="Y12" t="str">
         <v/>
       </c>
@@ -2487,53 +2619,53 @@
         <v/>
       </c>
       <c r="AC12" t="str">
+        <v/>
+      </c>
+      <c r="AD12">
+        <v>4</v>
+      </c>
+      <c r="AE12" t="str">
         <v>예시 옐로</v>
       </c>
-      <c r="AD12" t="str">
+      <c r="AF12" t="str">
         <v>다크 그레이</v>
       </c>
-      <c r="AE12" t="str">
+      <c r="AG12" t="str">
         <v>다크 그레이</v>
       </c>
-      <c r="AF12" t="str">
+      <c r="AH12" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG12" t="str">
+      <c r="AI12" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH12" t="str">
+      <c r="AJ12" t="str">
         <v>유광</v>
       </c>
-      <c r="AI12" t="str">
-        <v/>
-      </c>
-      <c r="AJ12">
+      <c r="AK12" t="str">
+        <v/>
+      </c>
+      <c r="AL12">
+        <v>3</v>
+      </c>
+      <c r="AM12">
         <v>19200</v>
       </c>
-      <c r="AK12">
+      <c r="AN12">
         <v>168</v>
       </c>
-      <c r="AL12" t="str">
-        <v/>
-      </c>
-      <c r="AM12">
+      <c r="AO12" t="str">
+        <v/>
+      </c>
+      <c r="AP12">
         <v>3.5</v>
       </c>
-      <c r="AN12" t="str">
+      <c r="AQ12" t="str">
         <v>디젤 · 토크컨버터 (예시)</v>
       </c>
-      <c r="AO12" t="str">
+      <c r="AR12" t="str">
         <v>측면 지상 점검</v>
       </c>
-      <c r="AP12" t="str">
-        <v/>
-      </c>
-      <c r="AQ12" t="str">
-        <v/>
-      </c>
-      <c r="AR12" t="str">
-        <v/>
-      </c>
       <c r="AS12" t="str">
         <v/>
       </c>
@@ -2541,45 +2673,57 @@
         <v/>
       </c>
       <c r="AU12" t="str">
+        <v/>
+      </c>
+      <c r="AV12" t="str">
+        <v/>
+      </c>
+      <c r="AW12" t="str">
+        <v/>
+      </c>
+      <c r="AX12">
+        <v>4</v>
+      </c>
+      <c r="AY12" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV12" t="str">
-        <v/>
-      </c>
-      <c r="AW12" t="str">
-        <v/>
-      </c>
-      <c r="AX12" t="str">
-        <v/>
-      </c>
-      <c r="AY12" t="str">
+      <c r="AZ12" t="str">
+        <v/>
+      </c>
+      <c r="BA12" t="str">
+        <v/>
+      </c>
+      <c r="BB12" t="str">
+        <v/>
+      </c>
+      <c r="BC12" t="str">
         <v>미검토</v>
       </c>
-      <c r="AZ12" t="str">
+      <c r="BD12" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA12" t="str">
+      <c r="BE12" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB12" t="str">
-        <v/>
-      </c>
-      <c r="BC12" t="str">
-        <v/>
-      </c>
-      <c r="BD12" t="str">
-        <v/>
-      </c>
-      <c r="BE12" t="str">
+      <c r="BF12" t="str">
+        <v/>
+      </c>
+      <c r="BG12" t="str">
+        <v/>
+      </c>
+      <c r="BH12" t="str">
+        <v/>
+      </c>
+      <c r="BI12" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF12" t="str">
+      <c r="BJ12" t="str">
         <v>Side; Front-Quarter; Cabin; CMF Detail</v>
       </c>
-      <c r="BG12" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH12" t="str">
+      <c r="BK12" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL12" t="str">
         <v>M0011</v>
       </c>
     </row>
@@ -2644,18 +2788,18 @@
       <c r="T13" t="str">
         <v>후방 경사 후드, 슬림 필러</v>
       </c>
-      <c r="U13" t="str">
+      <c r="U13">
+        <v>4</v>
+      </c>
+      <c r="V13" t="str">
         <v>넓음(전면 일체형)</v>
       </c>
-      <c r="V13" t="str">
+      <c r="W13" t="str">
         <v>슬림 A필러</v>
       </c>
-      <c r="W13" t="str">
+      <c r="X13" t="str">
         <v>전방·측방 양호</v>
       </c>
-      <c r="X13" t="str">
-        <v/>
-      </c>
       <c r="Y13" t="str">
         <v/>
       </c>
@@ -2669,53 +2813,53 @@
         <v/>
       </c>
       <c r="AC13" t="str">
+        <v/>
+      </c>
+      <c r="AD13">
+        <v>5</v>
+      </c>
+      <c r="AE13" t="str">
         <v>예시 실버</v>
       </c>
-      <c r="AD13" t="str">
+      <c r="AF13" t="str">
         <v>네이비</v>
       </c>
-      <c r="AE13" t="str">
+      <c r="AG13" t="str">
         <v>네이비</v>
       </c>
-      <c r="AF13" t="str">
+      <c r="AH13" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG13" t="str">
+      <c r="AI13" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH13" t="str">
+      <c r="AJ13" t="str">
         <v>반광</v>
       </c>
-      <c r="AI13" t="str">
-        <v/>
-      </c>
-      <c r="AJ13">
+      <c r="AK13" t="str">
+        <v/>
+      </c>
+      <c r="AL13">
+        <v>3</v>
+      </c>
+      <c r="AM13">
         <v>16800</v>
       </c>
-      <c r="AK13">
+      <c r="AN13">
         <v>150</v>
       </c>
-      <c r="AL13" t="str">
-        <v/>
-      </c>
-      <c r="AM13">
+      <c r="AO13" t="str">
+        <v/>
+      </c>
+      <c r="AP13">
         <v>3.2</v>
       </c>
-      <c r="AN13" t="str">
+      <c r="AQ13" t="str">
         <v>디젤 · 토크컨버터 (예시)</v>
       </c>
-      <c r="AO13" t="str">
+      <c r="AR13" t="str">
         <v>측면 지상 점검</v>
       </c>
-      <c r="AP13" t="str">
-        <v/>
-      </c>
-      <c r="AQ13" t="str">
-        <v/>
-      </c>
-      <c r="AR13" t="str">
-        <v/>
-      </c>
       <c r="AS13" t="str">
         <v/>
       </c>
@@ -2723,45 +2867,57 @@
         <v/>
       </c>
       <c r="AU13" t="str">
+        <v/>
+      </c>
+      <c r="AV13" t="str">
+        <v/>
+      </c>
+      <c r="AW13" t="str">
+        <v/>
+      </c>
+      <c r="AX13">
+        <v>3</v>
+      </c>
+      <c r="AY13" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV13" t="str">
-        <v/>
-      </c>
-      <c r="AW13" t="str">
-        <v/>
-      </c>
-      <c r="AX13" t="str">
-        <v/>
-      </c>
-      <c r="AY13" t="str">
+      <c r="AZ13" t="str">
+        <v/>
+      </c>
+      <c r="BA13" t="str">
+        <v/>
+      </c>
+      <c r="BB13" t="str">
+        <v/>
+      </c>
+      <c r="BC13" t="str">
         <v>미검토</v>
       </c>
-      <c r="AZ13" t="str">
+      <c r="BD13" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA13" t="str">
+      <c r="BE13" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB13" t="str">
-        <v/>
-      </c>
-      <c r="BC13" t="str">
-        <v/>
-      </c>
-      <c r="BD13" t="str">
-        <v/>
-      </c>
-      <c r="BE13" t="str">
+      <c r="BF13" t="str">
+        <v/>
+      </c>
+      <c r="BG13" t="str">
+        <v/>
+      </c>
+      <c r="BH13" t="str">
+        <v/>
+      </c>
+      <c r="BI13" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF13" t="str">
+      <c r="BJ13" t="str">
         <v>Side; Front-Quarter; Cabin</v>
       </c>
-      <c r="BG13" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH13" t="str">
+      <c r="BK13" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL13" t="str">
         <v>M0012</v>
       </c>
     </row>
@@ -2826,18 +2982,18 @@
       <c r="T14" t="str">
         <v>각진 볼륨</v>
       </c>
-      <c r="U14" t="str">
+      <c r="U14">
+        <v>3</v>
+      </c>
+      <c r="V14" t="str">
         <v>보통</v>
       </c>
-      <c r="V14" t="str">
+      <c r="W14" t="str">
         <v>일반 A필러</v>
       </c>
-      <c r="W14" t="str">
+      <c r="X14" t="str">
         <v>측방 보통</v>
       </c>
-      <c r="X14" t="str">
-        <v/>
-      </c>
       <c r="Y14" t="str">
         <v/>
       </c>
@@ -2851,53 +3007,53 @@
         <v/>
       </c>
       <c r="AC14" t="str">
+        <v/>
+      </c>
+      <c r="AD14">
+        <v>3</v>
+      </c>
+      <c r="AE14" t="str">
         <v>예시 블루</v>
       </c>
-      <c r="AD14" t="str">
+      <c r="AF14" t="str">
         <v>차콜</v>
       </c>
-      <c r="AE14" t="str">
+      <c r="AG14" t="str">
         <v>차콜</v>
       </c>
-      <c r="AF14" t="str">
+      <c r="AH14" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG14" t="str">
+      <c r="AI14" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH14" t="str">
+      <c r="AJ14" t="str">
         <v>유광</v>
       </c>
-      <c r="AI14" t="str">
-        <v/>
-      </c>
-      <c r="AJ14">
+      <c r="AK14" t="str">
+        <v/>
+      </c>
+      <c r="AL14">
+        <v>3</v>
+      </c>
+      <c r="AM14">
         <v>18900</v>
       </c>
-      <c r="AK14">
+      <c r="AN14">
         <v>164</v>
       </c>
-      <c r="AL14" t="str">
-        <v/>
-      </c>
-      <c r="AM14">
+      <c r="AO14" t="str">
+        <v/>
+      </c>
+      <c r="AP14">
         <v>3.4</v>
       </c>
-      <c r="AN14" t="str">
+      <c r="AQ14" t="str">
         <v>디젤 · 토크컨버터 (예시)</v>
       </c>
-      <c r="AO14" t="str">
+      <c r="AR14" t="str">
         <v>측면 + 상부 점검</v>
       </c>
-      <c r="AP14" t="str">
-        <v/>
-      </c>
-      <c r="AQ14" t="str">
-        <v/>
-      </c>
-      <c r="AR14" t="str">
-        <v/>
-      </c>
       <c r="AS14" t="str">
         <v/>
       </c>
@@ -2905,45 +3061,57 @@
         <v/>
       </c>
       <c r="AU14" t="str">
+        <v/>
+      </c>
+      <c r="AV14" t="str">
+        <v/>
+      </c>
+      <c r="AW14" t="str">
+        <v/>
+      </c>
+      <c r="AX14">
+        <v>3</v>
+      </c>
+      <c r="AY14" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV14" t="str">
-        <v/>
-      </c>
-      <c r="AW14" t="str">
-        <v/>
-      </c>
-      <c r="AX14" t="str">
-        <v/>
-      </c>
-      <c r="AY14" t="str">
+      <c r="AZ14" t="str">
+        <v/>
+      </c>
+      <c r="BA14" t="str">
+        <v/>
+      </c>
+      <c r="BB14" t="str">
+        <v/>
+      </c>
+      <c r="BC14" t="str">
         <v>확정</v>
       </c>
-      <c r="AZ14" t="str">
+      <c r="BD14" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA14" t="str">
+      <c r="BE14" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB14" t="str">
-        <v/>
-      </c>
-      <c r="BC14" t="str">
-        <v/>
-      </c>
-      <c r="BD14" t="str">
-        <v/>
-      </c>
-      <c r="BE14" t="str">
+      <c r="BF14" t="str">
+        <v/>
+      </c>
+      <c r="BG14" t="str">
+        <v/>
+      </c>
+      <c r="BH14" t="str">
+        <v/>
+      </c>
+      <c r="BI14" t="str">
         <v>(브라우저 보관 이미지); (브라우저 보관 이미지)</v>
       </c>
-      <c r="BF14" t="str">
+      <c r="BJ14" t="str">
         <v>Side; CMF Detail</v>
       </c>
-      <c r="BG14" t="str">
-        <v>v0.1-stage1</v>
-      </c>
-      <c r="BH14" t="str">
+      <c r="BK14" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL14" t="str">
         <v>M0013</v>
       </c>
     </row>
@@ -3008,18 +3176,18 @@
       <c r="T15" t="str">
         <v>라운드 후드</v>
       </c>
-      <c r="U15" t="str">
+      <c r="U15">
+        <v>3</v>
+      </c>
+      <c r="V15" t="str">
         <v>보통</v>
       </c>
-      <c r="V15" t="str">
+      <c r="W15" t="str">
         <v>일반 A필러</v>
       </c>
-      <c r="W15" t="str">
+      <c r="X15" t="str">
         <v>측방 보통</v>
       </c>
-      <c r="X15" t="str">
-        <v/>
-      </c>
       <c r="Y15" t="str">
         <v/>
       </c>
@@ -3033,53 +3201,53 @@
         <v/>
       </c>
       <c r="AC15" t="str">
+        <v/>
+      </c>
+      <c r="AD15">
+        <v>3</v>
+      </c>
+      <c r="AE15" t="str">
         <v>예시 그린</v>
       </c>
-      <c r="AD15" t="str">
+      <c r="AF15" t="str">
         <v>블랙</v>
       </c>
-      <c r="AE15" t="str">
+      <c r="AG15" t="str">
         <v>블랙</v>
       </c>
-      <c r="AF15" t="str">
+      <c r="AH15" t="str">
         <v>도장 강판 · 플라스틱 커버(예시)</v>
       </c>
-      <c r="AG15" t="str">
+      <c r="AI15" t="str">
         <v>솔리드 도장(예시)</v>
       </c>
-      <c r="AH15" t="str">
+      <c r="AJ15" t="str">
         <v>반광</v>
       </c>
-      <c r="AI15" t="str">
-        <v/>
-      </c>
-      <c r="AJ15">
+      <c r="AK15" t="str">
+        <v/>
+      </c>
+      <c r="AL15">
+        <v>2</v>
+      </c>
+      <c r="AM15">
         <v>15500</v>
       </c>
-      <c r="AK15">
+      <c r="AN15">
         <v>140</v>
       </c>
-      <c r="AL15" t="str">
-        <v/>
-      </c>
-      <c r="AM15">
+      <c r="AO15" t="str">
+        <v/>
+      </c>
+      <c r="AP15">
         <v>2.9</v>
       </c>
-      <c r="AN15" t="str">
+      <c r="AQ15" t="str">
         <v>디젤 · 토크컨버터 (예시)</v>
       </c>
-      <c r="AO15" t="str">
+      <c r="AR15" t="str">
         <v>측면 지상 점검</v>
       </c>
-      <c r="AP15" t="str">
-        <v/>
-      </c>
-      <c r="AQ15" t="str">
-        <v/>
-      </c>
-      <c r="AR15" t="str">
-        <v/>
-      </c>
       <c r="AS15" t="str">
         <v/>
       </c>
@@ -3087,51 +3255,257 @@
         <v/>
       </c>
       <c r="AU15" t="str">
+        <v/>
+      </c>
+      <c r="AV15" t="str">
+        <v/>
+      </c>
+      <c r="AW15" t="str">
+        <v/>
+      </c>
+      <c r="AX15">
+        <v>3</v>
+      </c>
+      <c r="AY15" t="str">
         <v>디자이너 입력</v>
       </c>
-      <c r="AV15" t="str">
-        <v/>
-      </c>
-      <c r="AW15" t="str">
-        <v/>
-      </c>
-      <c r="AX15" t="str">
-        <v/>
-      </c>
-      <c r="AY15" t="str">
+      <c r="AZ15" t="str">
+        <v/>
+      </c>
+      <c r="BA15" t="str">
+        <v/>
+      </c>
+      <c r="BB15" t="str">
+        <v/>
+      </c>
+      <c r="BC15" t="str">
         <v>미검토</v>
       </c>
-      <c r="AZ15" t="str">
+      <c r="BD15" t="str">
         <v>예시 데이터 — 실제 제품이 아닙니다</v>
       </c>
-      <c r="BA15" t="str">
+      <c r="BE15" t="str">
         <v>예시 입력자</v>
       </c>
-      <c r="BB15" t="str">
-        <v/>
-      </c>
-      <c r="BC15" t="str">
-        <v/>
-      </c>
-      <c r="BD15" t="str">
-        <v/>
-      </c>
-      <c r="BE15" t="str">
-        <v/>
-      </c>
       <c r="BF15" t="str">
         <v/>
       </c>
       <c r="BG15" t="str">
-        <v>v0.1-stage1</v>
+        <v/>
       </c>
       <c r="BH15" t="str">
+        <v/>
+      </c>
+      <c r="BI15" t="str">
+        <v/>
+      </c>
+      <c r="BJ15" t="str">
+        <v/>
+      </c>
+      <c r="BK15" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL15" t="str">
         <v>M0014</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Excavator</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Mecalac</v>
+      </c>
+      <c r="C16" t="str">
+        <v>예시-MW12</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Wheeled</v>
+      </c>
+      <c r="E16" t="str">
+        <v>MED</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v>예시 세대</v>
+      </c>
+      <c r="H16">
+        <v>2025</v>
+      </c>
+      <c r="I16" t="str">
+        <v>https://example.com/sample/예시-mw12</v>
+      </c>
+      <c r="J16" t="str">
+        <v>OEM 공식</v>
+      </c>
+      <c r="K16" t="str">
+        <v>예시 출처</v>
+      </c>
+      <c r="L16" t="str">
+        <v>2026-01-31</v>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v>1 공식 OEM</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Light &amp; open</v>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v>슬림 필러, 넓은 글라스</v>
+      </c>
+      <c r="U16">
+        <v>4</v>
+      </c>
+      <c r="V16" t="str">
+        <v>넓음(전면 일체형)</v>
+      </c>
+      <c r="W16" t="str">
+        <v>슬림 A필러</v>
+      </c>
+      <c r="X16" t="str">
+        <v>전방·측방 양호</v>
+      </c>
+      <c r="Y16" t="str">
+        <v/>
+      </c>
+      <c r="Z16" t="str">
+        <v/>
+      </c>
+      <c r="AA16" t="str">
+        <v/>
+      </c>
+      <c r="AB16" t="str">
+        <v/>
+      </c>
+      <c r="AC16" t="str">
+        <v/>
+      </c>
+      <c r="AD16">
+        <v>4</v>
+      </c>
+      <c r="AE16" t="str">
+        <v>예시 레드</v>
+      </c>
+      <c r="AF16" t="str">
+        <v>화이트</v>
+      </c>
+      <c r="AG16" t="str">
+        <v>화이트</v>
+      </c>
+      <c r="AH16" t="str">
+        <v>도장 강판 · 플라스틱 커버(예시)</v>
+      </c>
+      <c r="AI16" t="str">
+        <v>솔리드 도장(예시)</v>
+      </c>
+      <c r="AJ16" t="str">
+        <v>유광</v>
+      </c>
+      <c r="AK16" t="str">
+        <v/>
+      </c>
+      <c r="AL16">
+        <v>3</v>
+      </c>
+      <c r="AM16">
+        <v>11900</v>
+      </c>
+      <c r="AN16">
+        <v>85</v>
+      </c>
+      <c r="AO16" t="str">
+        <v/>
+      </c>
+      <c r="AP16">
+        <v>0.4</v>
+      </c>
+      <c r="AQ16" t="str">
+        <v>디젤 (예시)</v>
+      </c>
+      <c r="AR16" t="str">
+        <v>측면 지상 점검</v>
+      </c>
+      <c r="AS16" t="str">
+        <v/>
+      </c>
+      <c r="AT16" t="str">
+        <v/>
+      </c>
+      <c r="AU16" t="str">
+        <v/>
+      </c>
+      <c r="AV16" t="str">
+        <v/>
+      </c>
+      <c r="AW16" t="str">
+        <v/>
+      </c>
+      <c r="AX16">
+        <v>3</v>
+      </c>
+      <c r="AY16" t="str">
+        <v>디자이너 입력</v>
+      </c>
+      <c r="AZ16" t="str">
+        <v/>
+      </c>
+      <c r="BA16" t="str">
+        <v/>
+      </c>
+      <c r="BB16" t="str">
+        <v/>
+      </c>
+      <c r="BC16" t="str">
+        <v>미검토</v>
+      </c>
+      <c r="BD16" t="str">
+        <v>예시 데이터 — 실제 제품이 아닙니다</v>
+      </c>
+      <c r="BE16" t="str">
+        <v>예시 입력자</v>
+      </c>
+      <c r="BF16" t="str">
+        <v/>
+      </c>
+      <c r="BG16" t="str">
+        <v/>
+      </c>
+      <c r="BH16" t="str">
+        <v/>
+      </c>
+      <c r="BI16" t="str">
+        <v>(브라우저 보관 이미지); (브라우저 보관 이미지); (브라우저 보관 이미지)</v>
+      </c>
+      <c r="BJ16" t="str">
+        <v>Side; Front-Quarter; Cabin</v>
+      </c>
+      <c r="BK16" t="str">
+        <v>v0.2-stage1</v>
+      </c>
+      <c r="BL16" t="str">
+        <v>M0015</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:BH15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:BL16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>